<commit_message>
Utiliser Qt dans les classes
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\groupe19\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE869F4-BE5A-493F-AEF2-AF7F930D88EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888F8782-D8B3-438D-9AA1-BB82F18527A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -279,7 +279,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -940,16 +940,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>358140</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>350520</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1245,7 +1245,7 @@
   <cols>
     <col min="2" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.5546875" customWidth="1"/>
-    <col min="6" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -1268,7 +1268,9 @@
       <c r="G1" s="4">
         <v>45804</v>
       </c>
-      <c r="H1" s="3"/>
+      <c r="H1" s="5">
+        <v>45804</v>
+      </c>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
@@ -1333,7 +1335,9 @@
       <c r="G3" s="6">
         <v>1</v>
       </c>
-      <c r="H3" s="6"/>
+      <c r="H3" s="6">
+        <v>2</v>
+      </c>
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
@@ -1342,7 +1346,7 @@
       <c r="N3" s="6"/>
       <c r="O3" s="6">
         <f>SUM(B3:N3)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -1375,7 +1379,7 @@
       </c>
       <c r="H4" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I4" s="6">
         <f t="shared" si="0"/>
@@ -1403,7 +1407,7 @@
       </c>
       <c r="O4" s="6">
         <f>SUM(B4:N4)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Afficher dans Qdebug() les recettes XML chargées
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888F8782-D8B3-438D-9AA1-BB82F18527A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27FB783F-78D9-4B1E-9602-621C480BC55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -279,7 +279,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1245,7 +1245,7 @@
   <cols>
     <col min="2" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.5546875" customWidth="1"/>
-    <col min="6" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -1271,7 +1271,9 @@
       <c r="H1" s="5">
         <v>45804</v>
       </c>
-      <c r="I1" s="3"/>
+      <c r="I1" s="5">
+        <v>45811</v>
+      </c>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
@@ -1338,7 +1340,9 @@
       <c r="H3" s="6">
         <v>2</v>
       </c>
-      <c r="I3" s="6"/>
+      <c r="I3" s="6">
+        <v>1</v>
+      </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
@@ -1346,7 +1350,7 @@
       <c r="N3" s="6"/>
       <c r="O3" s="6">
         <f>SUM(B3:N3)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -1383,7 +1387,7 @@
       </c>
       <c r="I4" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" s="6">
         <f t="shared" si="0"/>
@@ -1407,7 +1411,7 @@
       </c>
       <c r="O4" s="6">
         <f>SUM(B4:N4)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Afficher et éditer dans l'application Supression du dossier buil qui n'a pas d'intérêt à être déposer
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27FB783F-78D9-4B1E-9602-621C480BC55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572405A3-0D7B-41A9-B35F-BE0B1F774659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuille de temps" sheetId="1" r:id="rId1"/>
+    <sheet name="Heures cumulées" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Chadi</t>
   </si>
@@ -52,11 +53,26 @@
   <si>
     <t>Session individuelle</t>
   </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Chadi cumulé</t>
+  </si>
+  <si>
+    <t>Thomas cumulé</t>
+  </si>
+  <si>
+    <t>Total cumulé</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -113,14 +129,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -255,9 +275,66 @@
               </c:ext>
             </c:extLst>
           </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:separator>
+</c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$2:$A$3</c:f>
+              <c:f>'Feuille de temps'!$A$2:$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -271,15 +348,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$O$2:$O$3</c:f>
+              <c:f>'Feuille de temps'!$O$2:$O$3</c:f>
               <c:numCache>
-                <c:formatCode>0</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
+                <c:pt idx="0" formatCode="0">
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -377,7 +454,1457 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="fr-FR"/>
+              <a:t>Répartition du travail par session</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Feuille de temps'!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Chadi</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Feuille de temps'!$B$1:$I$1</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>45782</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45783</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45790</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45811</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Feuille de temps'!$B$2:$I$2</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-EB98-4DFE-8007-B305B6A0E767}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Feuille de temps'!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Thomas</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Feuille de temps'!$B$1:$I$1</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>45782</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45783</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45790</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45811</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Feuille de temps'!$B$3:$I$3</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="0.0">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-EB98-4DFE-8007-B305B6A0E767}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1382641760"/>
+        <c:axId val="1382631200"/>
+      </c:barChart>
+      <c:dateAx>
+        <c:axId val="1382641760"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="fr-FR"/>
+                  <a:t>Sessions</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="fr-FR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1382631200"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+        <c:baseTimeUnit val="days"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="1382631200"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="fr-FR"/>
+                  <a:t>Heures de travail</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="fr-FR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1382641760"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="fr-FR"/>
+              <a:t>Progression</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="fr-FR" baseline="0"/>
+              <a:t> cumulative du projet</a:t>
+            </a:r>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Heures cumulées'!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Chadi cumulé</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Heures cumulées'!$A$2:$A$23</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>45782</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45783</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45790</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45811</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>45820</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Heures cumulées'!$D$2:$D$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9FDA-4D4A-B62C-896704D1A0D1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Heures cumulées'!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Thomas cumulé</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Heures cumulées'!$A$2:$A$23</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>45782</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45783</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45790</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45811</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>45820</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Heures cumulées'!$E$2:$E$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9FDA-4D4A-B62C-896704D1A0D1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Heures cumulées'!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total cumulé</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Heures cumulées'!$A$2:$A$23</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>45782</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45783</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45790</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45804</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45811</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>45820</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Heures cumulées'!$F$2:$F$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="22"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>29</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-9FDA-4D4A-B62C-896704D1A0D1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1454879536"/>
+        <c:axId val="1454889616"/>
+      </c:lineChart>
+      <c:dateAx>
+        <c:axId val="1454879536"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="fr-FR"/>
+                  <a:t>Timeline</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="fr-FR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1454889616"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+        <c:baseTimeUnit val="days"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="1454889616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="fr-FR"/>
+                  <a:t>Heures cumulées</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="fr-FR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1454879536"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -936,20 +2463,1028 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>350520</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>662940</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>125730</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -957,6 +3492,83 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A9E3A4D-B8E9-7422-2A8F-45CB76A53CFF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Graphique 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEEFC16E-6200-104B-B68B-33972A5B545F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>148590</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>148590</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Graphique 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52F72CD5-A640-6CE7-B145-8020B2F4537A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1249,180 +3861,539 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="3"/>
-      <c r="B1" s="4">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3">
         <v>45782</v>
       </c>
-      <c r="C1" s="4">
+      <c r="C1" s="3">
         <v>45783</v>
       </c>
-      <c r="D1" s="4">
+      <c r="D1" s="3">
         <v>45789</v>
       </c>
-      <c r="E1" s="4">
+      <c r="E1" s="3">
         <v>45790</v>
       </c>
-      <c r="F1" s="5">
+      <c r="F1" s="4">
         <v>45799</v>
       </c>
-      <c r="G1" s="4">
+      <c r="G1" s="3">
         <v>45804</v>
       </c>
-      <c r="H1" s="5">
+      <c r="H1" s="4">
         <v>45804</v>
       </c>
-      <c r="I1" s="5">
+      <c r="I1" s="4">
         <v>45811</v>
       </c>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3" t="s">
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <v>2</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>2</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="5">
         <v>2</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="5">
         <v>2</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6">
+      <c r="F2" s="5"/>
+      <c r="G2" s="5">
         <v>1</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5">
         <f>SUM(B2:N2)</f>
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="5">
         <v>2</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>2</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <v>2</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>2</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>2</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="5">
         <v>1</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="6">
-        <v>1</v>
-      </c>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6">
+      <c r="I3" s="8">
+        <v>3</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="8">
         <f>SUM(B3:N3)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <f>SUM(B2:B3)</f>
         <v>4</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <f t="shared" ref="C4:N4" si="0">SUM(C2:C3)</f>
         <v>4</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J4" s="6">
+        <v>3</v>
+      </c>
+      <c r="J4" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="8">
         <f>SUM(B4:N4)</f>
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B11" s="1" t="s">
+    <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B11" s="6" t="s">
         <v>4</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A4437B1-41E4-4615-925C-54B5BCB12A56}">
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="7">
+        <v>45782</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <f>D2+E2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="7">
+        <v>45783</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <f>D2+B3</f>
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <f>E2+C3</f>
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F17" si="0">D3+E3</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>45789</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D17" si="1">D3+B4</f>
+        <v>6</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E17" si="2">E3+C4</f>
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="7">
+        <v>45790</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>45799</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="7">
+        <v>45804</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
+        <v>45804</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
+        <v>45811</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="7"/>
+      <c r="D10">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7"/>
+      <c r="D11">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="7"/>
+      <c r="D12">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="7"/>
+      <c r="D13">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="7"/>
+      <c r="D14">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="7"/>
+      <c r="D15">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="7"/>
+      <c r="D16">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
+        <v>45820</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="7"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finaliser traduction/Ajouter recette La fonction chargerXML ne charge que la première recette.
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572405A3-0D7B-41A9-B35F-BE0B1F774659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF547285-2E7D-4FC1-B94A-80DFF49C6FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille de temps" sheetId="1" r:id="rId1"/>
@@ -129,13 +129,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -352,11 +351,11 @@
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0" formatCode="0">
+                <c:pt idx="0">
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -591,7 +590,7 @@
             <c:numRef>
               <c:f>'Feuille de temps'!$B$2:$I$2</c:f>
               <c:numCache>
-                <c:formatCode>0</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
@@ -678,7 +677,7 @@
             <c:numRef>
               <c:f>'Feuille de temps'!$B$3:$I$3</c:f>
               <c:numCache>
-                <c:formatCode>0</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
@@ -701,7 +700,7 @@
                 <c:pt idx="6">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="7" formatCode="0.0">
+                <c:pt idx="7">
                   <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
@@ -907,7 +906,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1166,6 +1165,12 @@
                 <c:pt idx="7">
                   <c:v>45811</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45813</c:v>
+                </c:pt>
                 <c:pt idx="15">
                   <c:v>45820</c:v>
                 </c:pt>
@@ -1304,6 +1309,12 @@
                 <c:pt idx="7">
                   <c:v>45811</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45813</c:v>
+                </c:pt>
                 <c:pt idx="15">
                   <c:v>45820</c:v>
                 </c:pt>
@@ -1341,28 +1352,28 @@
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>16</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>18</c:v>
+                  <c:v>22.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1442,6 +1453,12 @@
                 <c:pt idx="7">
                   <c:v>45811</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45813</c:v>
+                </c:pt>
                 <c:pt idx="15">
                   <c:v>45820</c:v>
                 </c:pt>
@@ -1479,28 +1496,28 @@
                   <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>25</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>29</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3855,9 +3872,12 @@
   <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.5546875" customWidth="1"/>
-    <col min="6" max="9" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.77734375" customWidth="1"/>
+    <col min="20" max="21" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -3886,8 +3906,12 @@
       <c r="I1" s="4">
         <v>45811</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
+      <c r="J1" s="3">
+        <v>45813</v>
+      </c>
+      <c r="K1" s="4">
+        <v>45813</v>
+      </c>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
@@ -3899,30 +3923,30 @@
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="7">
         <v>2</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="7">
         <v>2</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="7">
         <v>2</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="7">
         <v>2</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5">
+      <c r="F2" s="7"/>
+      <c r="G2" s="7">
         <v>1</v>
       </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5">
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7">
         <f>SUM(B2:N2)</f>
         <v>9</v>
       </c>
@@ -3931,99 +3955,103 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="7">
         <v>2</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="7">
         <v>2</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="7">
         <v>2</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="7">
         <v>2</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="7">
         <v>2</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="7">
         <v>1</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="7">
         <v>2</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="7">
         <v>3</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="8">
+      <c r="J3" s="7">
+        <v>2</v>
+      </c>
+      <c r="K3" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7">
         <f>SUM(B3:N3)</f>
-        <v>16</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="7">
         <f>SUM(B2:B3)</f>
         <v>4</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="7">
         <f t="shared" ref="C4:N4" si="0">SUM(C2:C3)</f>
         <v>4</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="7">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="7">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="7">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="7">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="7">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="7">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="7">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="K4" s="7">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="L4" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K4" s="5">
+      <c r="M4" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L4" s="5">
+      <c r="N4" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M4" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="N4" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O4" s="8">
+      <c r="O4" s="7">
         <f>SUM(B4:N4)</f>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -4032,7 +4060,7 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -4068,7 +4096,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="7">
+      <c r="A2" s="6">
         <v>45782</v>
       </c>
       <c r="B2">
@@ -4089,7 +4117,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7">
+      <c r="A3" s="6">
         <v>45783</v>
       </c>
       <c r="B3">
@@ -4112,7 +4140,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="7">
+      <c r="A4" s="6">
         <v>45789</v>
       </c>
       <c r="B4">
@@ -4135,7 +4163,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="7">
+      <c r="A5" s="6">
         <v>45790</v>
       </c>
       <c r="B5">
@@ -4158,7 +4186,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>45799</v>
       </c>
       <c r="B6">
@@ -4181,7 +4209,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>45804</v>
       </c>
       <c r="B7">
@@ -4204,7 +4232,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>45804</v>
       </c>
       <c r="B8">
@@ -4227,7 +4255,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <v>45811</v>
       </c>
       <c r="B9">
@@ -4250,112 +4278,122 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
+      <c r="A10" s="6">
+        <v>45813</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
       <c r="D10">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E10">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F10">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
+      <c r="A11" s="6">
+        <v>45813</v>
+      </c>
+      <c r="C11">
+        <v>2.5</v>
+      </c>
       <c r="D11">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E11">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>20.5</v>
       </c>
       <c r="F11">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
+      <c r="A12" s="6"/>
       <c r="D12">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E12">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>20.5</v>
       </c>
       <c r="F12">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
+      <c r="A13" s="6"/>
       <c r="D13">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>20.5</v>
       </c>
       <c r="F13">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
+      <c r="A14" s="6"/>
       <c r="D14">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>20.5</v>
       </c>
       <c r="F14">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+      <c r="A15" s="6"/>
       <c r="D15">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>20.5</v>
       </c>
       <c r="F15">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
+      <c r="A16" s="6"/>
       <c r="D16">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E16">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>20.5</v>
       </c>
       <c r="F16">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="7">
+      <c r="A17" s="6">
         <v>45820</v>
       </c>
       <c r="B17">
@@ -4370,30 +4408,30 @@
       </c>
       <c r="E17">
         <f t="shared" si="2"/>
-        <v>18</v>
+        <v>22.5</v>
       </c>
       <c r="F17">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
+      <c r="A18" s="6"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
+      <c r="A19" s="6"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
+      <c r="A20" s="6"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
+      <c r="A21" s="6"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="7"/>
+      <c r="A22" s="6"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="7"/>
+      <c r="A23" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Ajouter heures dernière session session (ajout images, dark mode)
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -1,18 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5011F503-4A3D-4076-8E3F-D917BFED5116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille de temps" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Heures cumulées" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Feuille de temps" sheetId="1" r:id="rId1"/>
+    <sheet name="Heures cumulées" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -23,88 +40,47 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
-    <t xml:space="preserve">Total</t>
+    <t>Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Chadi</t>
+    <t>Chadi</t>
   </si>
   <si>
-    <t xml:space="preserve">Thomas</t>
+    <t>Thomas</t>
   </si>
   <si>
-    <t xml:space="preserve">Cours</t>
+    <t>Cours</t>
   </si>
   <si>
-    <t xml:space="preserve">Session individuelle</t>
+    <t>Session individuelle</t>
   </si>
   <si>
-    <t xml:space="preserve">Date</t>
+    <t>Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Chadi cumulé</t>
+    <t>Chadi cumulé</t>
   </si>
   <si>
-    <t xml:space="preserve">Thomas cumulé</t>
+    <t>Thomas cumulé</t>
   </si>
   <si>
-    <t xml:space="preserve">Total cumulé</t>
+    <t>Total cumulé</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF595959"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF404040"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF595959"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF595959"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -128,88 +104,49 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -268,15 +205,33 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF404040"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:lang val="en-US"/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -285,7 +240,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" lang="fr-FR" sz="1400" spc="-1" strike="noStrike">
+              <a:defRPr lang="fr-FR" sz="1400" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -293,7 +248,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="0" lang="fr-FR" sz="1400" spc="-1" strike="noStrike">
+              <a:rPr lang="fr-FR" sz="1400" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -314,6 +269,7 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
+      <c:layout/>
       <c:pieChart>
         <c:varyColors val="1"/>
         <c:ser>
@@ -321,58 +277,69 @@
           <c:order val="0"/>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="5b9bd5"/>
+              <a:srgbClr val="5B9BD5"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
             </a:ln>
           </c:spPr>
-          <c:explosion val="0"/>
           <c:dPt>
             <c:idx val="0"/>
+            <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="5b9bd5"/>
+                <a:srgbClr val="5B9BD5"/>
               </a:solidFill>
               <a:ln w="19080">
                 <a:solidFill>
-                  <a:srgbClr val="ffffff"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:round/>
               </a:ln>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-CA7F-4612-9881-F92DD63E748B}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
+            <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="ed7d31"/>
+                <a:srgbClr val="ED7D31"/>
               </a:solidFill>
               <a:ln w="19080">
                 <a:solidFill>
-                  <a:srgbClr val="ffffff"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:round/>
               </a:ln>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-CA7F-4612-9881-F92DD63E748B}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
-            <c:numFmt formatCode="0.0" sourceLinked="1"/>
             <c:dLbl>
               <c:idx val="0"/>
-              <c:numFmt formatCode="0.0" sourceLinked="1"/>
+              <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
-                    <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
                         <a:srgbClr val="404040"/>
                       </a:solidFill>
                       <a:latin typeface="Calibri"/>
                     </a:defRPr>
                   </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
@@ -381,24 +348,29 @@
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>
-</c:separator>
+              <c:showBubbleSize val="1"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-CA7F-4612-9881-F92DD63E748B}"/>
+                </c:ext>
+              </c:extLst>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
-              <c:numFmt formatCode="0.0" sourceLinked="1"/>
+              <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
-                    <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                    <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                       <a:solidFill>
                         <a:srgbClr val="404040"/>
                       </a:solidFill>
                       <a:latin typeface="Calibri"/>
                     </a:defRPr>
                   </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
                 </a:p>
               </c:txPr>
               <c:dLblPos val="bestFit"/>
@@ -407,21 +379,33 @@
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="1"/>
-              <c:separator>
-</c:separator>
+              <c:showBubbleSize val="1"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-CA7F-4612-9881-F92DD63E748B}"/>
+                </c:ext>
+              </c:extLst>
             </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                  <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="404040"/>
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="bestFit"/>
@@ -430,9 +414,13 @@
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="1"/>
+            <c:showBubbleSize val="1"/>
             <c:separator>
 </c:separator>
             <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -452,18 +440,32 @@
             <c:numRef>
               <c:f>'Feuille de temps'!$O$2:$O$3</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>20.5</c:v>
+                  <c:v>25.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-CA7F-4612-9881-F92DD63E748B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
       <c:spPr>
@@ -487,37 +489,46 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+            <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="595959"/>
               </a:solidFill>
               <a:latin typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
   </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:lang val="en-US"/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -526,7 +537,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" lang="fr-FR" sz="1400" spc="-1" strike="noStrike">
+              <a:defRPr lang="fr-FR" sz="1400" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -534,7 +545,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="0" lang="fr-FR" sz="1400" spc="-1" strike="noStrike">
+              <a:rPr lang="fr-FR" sz="1400" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -555,6 +566,7 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
+      <c:layout/>
       <c:barChart>
         <c:barDir val="bar"/>
         <c:grouping val="stacked"/>
@@ -575,7 +587,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="5b9bd5"/>
+              <a:srgbClr val="5B9BD5"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -583,18 +595,26 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="ctr"/>
@@ -603,8 +623,9 @@
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
-            <c:showLeaderLines val="1"/>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -618,28 +639,28 @@
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>05/05/2025</c:v>
+                  <c:v>45782</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>06/05/2025</c:v>
+                  <c:v>45783</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12/05/2025</c:v>
+                  <c:v>45789</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13/05/2025</c:v>
+                  <c:v>45790</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22/05/2025</c:v>
+                  <c:v>45799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/06/2025</c:v>
+                  <c:v>45811</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -648,7 +669,7 @@
             <c:numRef>
               <c:f>'Feuille de temps'!$B$2:$I$2</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
@@ -668,6 +689,11 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2576-438B-8046-3FA84E2B1867}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -685,7 +711,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ed7d31"/>
+              <a:srgbClr val="ED7D31"/>
             </a:solidFill>
             <a:ln w="0">
               <a:noFill/>
@@ -693,18 +719,26 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="ctr"/>
@@ -713,8 +747,9 @@
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
-            <c:showLeaderLines val="1"/>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -728,28 +763,28 @@
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>05/05/2025</c:v>
+                  <c:v>45782</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>06/05/2025</c:v>
+                  <c:v>45783</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12/05/2025</c:v>
+                  <c:v>45789</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13/05/2025</c:v>
+                  <c:v>45790</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22/05/2025</c:v>
+                  <c:v>45799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/06/2025</c:v>
+                  <c:v>45811</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -758,7 +793,7 @@
             <c:numRef>
               <c:f>'Feuille de temps'!$B$3:$I$3</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
@@ -787,7 +822,20 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-2576-438B-8046-3FA84E2B1867}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
         <c:axId val="2896834"/>
@@ -799,7 +847,7 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
         <c:title>
           <c:tx>
             <c:rich>
@@ -807,7 +855,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -815,7 +863,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:rPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -841,7 +889,7 @@
         <c:spPr>
           <a:ln w="9360">
             <a:solidFill>
-              <a:srgbClr val="d9d9d9"/>
+              <a:srgbClr val="D9D9D9"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -851,13 +899,14 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+              <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="48088748"/>
@@ -865,7 +914,6 @@
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
         <c:baseTimeUnit val="days"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
         <c:axId val="48088748"/>
@@ -873,12 +921,12 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="d9d9d9"/>
+                <a:srgbClr val="D9D9D9"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -891,7 +939,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -899,7 +947,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:rPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -932,13 +980,14 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+              <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="2896834"/>
@@ -966,37 +1015,46 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+            <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="595959"/>
               </a:solidFill>
               <a:latin typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
   </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:lang val="en-US"/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1005,7 +1063,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" lang="fr-FR" sz="1400" spc="-1" strike="noStrike">
+              <a:defRPr lang="fr-FR" sz="1400" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -1013,7 +1071,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="0" lang="fr-FR" sz="1400" spc="-1" strike="noStrike">
+              <a:rPr lang="fr-FR" sz="1400" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -1034,6 +1092,7 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
+      <c:layout/>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -1052,12 +1111,9 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="5b9bd5"/>
-            </a:solidFill>
-            <a:ln cap="rnd" w="28440">
+            <a:ln w="28440" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="5b9bd5"/>
+                <a:srgbClr val="5B9BD5"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1067,23 +1123,31 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="5b9bd5"/>
+                <a:srgbClr val="5B9BD5"/>
               </a:solidFill>
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="r"/>
@@ -1092,8 +1156,9 @@
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
-            <c:showLeaderLines val="1"/>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -1107,70 +1172,40 @@
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>05/05/2025</c:v>
+                  <c:v>45782</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>06/05/2025</c:v>
+                  <c:v>45783</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12/05/2025</c:v>
+                  <c:v>45789</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13/05/2025</c:v>
+                  <c:v>45790</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22/05/2025</c:v>
+                  <c:v>45799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/06/2025</c:v>
+                  <c:v>45811</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>05/06/2025</c:v>
+                  <c:v>45813</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>05/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v/>
+                  <c:v>45813</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>10/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v/>
+                  <c:v>45818</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>12/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v/>
+                  <c:v>45820</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1233,6 +1268,11 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-566D-44AC-9121-29448D12FE55}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -1249,12 +1289,9 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="ed7d31"/>
-            </a:solidFill>
-            <a:ln cap="rnd" w="28440">
+            <a:ln w="28440" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="ed7d31"/>
+                <a:srgbClr val="ED7D31"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1264,23 +1301,31 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="ed7d31"/>
+                <a:srgbClr val="ED7D31"/>
               </a:solidFill>
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="r"/>
@@ -1289,8 +1334,9 @@
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
-            <c:showLeaderLines val="1"/>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -1304,70 +1350,40 @@
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>05/05/2025</c:v>
+                  <c:v>45782</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>06/05/2025</c:v>
+                  <c:v>45783</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12/05/2025</c:v>
+                  <c:v>45789</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13/05/2025</c:v>
+                  <c:v>45790</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22/05/2025</c:v>
+                  <c:v>45799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/06/2025</c:v>
+                  <c:v>45811</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>05/06/2025</c:v>
+                  <c:v>45813</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>05/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v/>
+                  <c:v>45813</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>10/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v/>
+                  <c:v>45818</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>12/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v/>
+                  <c:v>45820</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1415,21 +1431,26 @@
                   <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>20.5</c:v>
+                  <c:v>23.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>20.5</c:v>
+                  <c:v>23.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>20.5</c:v>
+                  <c:v>23.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>22.5</c:v>
+                  <c:v>25.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-566D-44AC-9121-29448D12FE55}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -1446,10 +1467,7 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:ln cap="rnd" w="38160">
+            <a:ln w="38160" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1466,18 +1484,26 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="r"/>
@@ -1486,8 +1512,9 @@
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
             <c:separator>; </c:separator>
-            <c:showLeaderLines val="1"/>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -1501,70 +1528,40 @@
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>05/05/2025</c:v>
+                  <c:v>45782</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>06/05/2025</c:v>
+                  <c:v>45783</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12/05/2025</c:v>
+                  <c:v>45789</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13/05/2025</c:v>
+                  <c:v>45790</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22/05/2025</c:v>
+                  <c:v>45799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>27/05/2025</c:v>
+                  <c:v>45804</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/06/2025</c:v>
+                  <c:v>45811</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>05/06/2025</c:v>
+                  <c:v>45813</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>05/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v/>
+                  <c:v>45813</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>10/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v/>
+                  <c:v>45818</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>12/06/2025</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v/>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v/>
+                  <c:v>45820</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1612,22 +1609,35 @@
                   <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>35.5</c:v>
+                  <c:v>38.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>35.5</c:v>
+                  <c:v>38.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>35.5</c:v>
+                  <c:v>38.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>39.5</c:v>
+                  <c:v>42.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-566D-44AC-9121-29448D12FE55}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:hiLowLines>
           <c:spPr>
             <a:ln w="0">
@@ -1636,6 +1646,7 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
+        <c:smooth val="0"/>
         <c:axId val="97318348"/>
         <c:axId val="88727794"/>
       </c:lineChart>
@@ -1653,7 +1664,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -1661,7 +1672,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:rPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -1687,7 +1698,7 @@
         <c:spPr>
           <a:ln w="9360">
             <a:solidFill>
-              <a:srgbClr val="d9d9d9"/>
+              <a:srgbClr val="D9D9D9"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -1697,13 +1708,14 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+              <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88727794"/>
@@ -1711,7 +1723,6 @@
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
         <c:baseTimeUnit val="days"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
         <c:axId val="88727794"/>
@@ -1724,7 +1735,7 @@
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="d9d9d9"/>
+                <a:srgbClr val="D9D9D9"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1737,7 +1748,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -1745,7 +1756,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr b="0" lang="fr-FR" sz="1000" spc="-1" strike="noStrike">
+                  <a:rPr lang="fr-FR" sz="1000" b="0" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="595959"/>
                     </a:solidFill>
@@ -1778,13 +1789,14 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+              <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="97318348"/>
@@ -1812,35 +1824,42 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+            <a:defRPr sz="900" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="595959"/>
               </a:solidFill>
               <a:latin typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="ffffff"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
   </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1854,14 +1873,20 @@
       <xdr:row>26</xdr:row>
       <xdr:rowOff>125280</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame>
+    <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="0" name="Graphique 1"/>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="160200" y="2586960"/>
-        <a:ext cx="4172400" cy="2424600"/>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1880,18 +1905,24 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>495000</xdr:colOff>
+      <xdr:colOff>266400</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>11160</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame>
+    <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1" name="Graphique 3"/>
+        <xdr:cNvPr id="3" name="Graphique 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5578560" y="2545200"/>
-        <a:ext cx="4952520" cy="2714400"/>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1905,7 +1936,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
@@ -1919,14 +1950,20 @@
       <xdr:row>21</xdr:row>
       <xdr:rowOff>148320</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame>
+    <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Graphique 2"/>
+        <xdr:cNvPr id="2" name="Graphique 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="4686480" y="1234440"/>
-        <a:ext cx="4244040" cy="2714400"/>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1939,594 +1976,909 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O11"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="3" style="0" width="10.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10.77"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="10" width="10.5546875" customWidth="1"/>
+    <col min="11" max="11" width="10.77734375" customWidth="1"/>
+    <col min="12" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="2" t="n">
+      <c r="B1" s="2">
         <v>45782</v>
       </c>
-      <c r="C1" s="2" t="n">
+      <c r="C1" s="2">
         <v>45783</v>
       </c>
-      <c r="D1" s="2" t="n">
+      <c r="D1" s="2">
         <v>45789</v>
       </c>
-      <c r="E1" s="2" t="n">
+      <c r="E1" s="2">
         <v>45790</v>
       </c>
-      <c r="F1" s="3" t="n">
+      <c r="F1" s="3">
         <v>45799</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="G1" s="2">
         <v>45804</v>
       </c>
-      <c r="H1" s="3" t="n">
+      <c r="H1" s="3">
         <v>45804</v>
       </c>
-      <c r="I1" s="3" t="n">
+      <c r="I1" s="3">
         <v>45811</v>
       </c>
-      <c r="J1" s="2" t="n">
+      <c r="J1" s="2">
         <v>45813</v>
       </c>
-      <c r="K1" s="3" t="n">
+      <c r="K1" s="3">
         <v>45813</v>
       </c>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
+      <c r="L1" s="3">
+        <v>45818</v>
+      </c>
+      <c r="M1" s="2">
+        <v>45820</v>
+      </c>
       <c r="N1" s="1"/>
       <c r="O1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" s="4" t="n">
+      <c r="B2" s="4">
+        <v>2</v>
+      </c>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4">
         <v>2</v>
       </c>
       <c r="F2" s="4"/>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="4">
         <v>1</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
+      <c r="L2" s="4">
+        <v>6</v>
+      </c>
+      <c r="M2" s="4">
+        <v>2</v>
+      </c>
       <c r="N2" s="4"/>
-      <c r="O2" s="4" t="n">
-        <f aca="false">SUM(B2:N2)</f>
-        <v>9</v>
+      <c r="O2" s="4">
+        <f>SUM(B2:N2)</f>
+        <v>17</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" s="4" t="n">
+      <c r="B3" s="4">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4">
+        <v>2</v>
+      </c>
+      <c r="G3" s="4">
         <v>1</v>
       </c>
-      <c r="H3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" s="4" t="n">
+      <c r="H3" s="4">
+        <v>2</v>
+      </c>
+      <c r="I3" s="4">
         <v>3</v>
       </c>
-      <c r="J3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" s="4" t="n">
+      <c r="J3" s="4">
+        <v>2</v>
+      </c>
+      <c r="K3" s="4">
         <v>2.5</v>
       </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
+      <c r="L3" s="4">
+        <v>3</v>
+      </c>
+      <c r="M3" s="4">
+        <v>2</v>
+      </c>
       <c r="N3" s="4"/>
-      <c r="O3" s="4" t="n">
-        <f aca="false">SUM(B3:N3)</f>
-        <v>20.5</v>
+      <c r="O3" s="4">
+        <f>SUM(B3:N3)</f>
+        <v>25.5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="4" t="n">
-        <f aca="false">SUM(B2:B3)</f>
+      <c r="B4" s="4">
+        <f t="shared" ref="B4:N4" si="0">SUM(B2:B3)</f>
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="n">
-        <f aca="false">SUM(C2:C3)</f>
+      <c r="C4" s="4">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <f aca="false">SUM(D2:D3)</f>
+      <c r="D4" s="4">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <f aca="false">SUM(E2:E3)</f>
+      <c r="E4" s="4">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F4" s="4" t="n">
-        <f aca="false">SUM(F2:F3)</f>
-        <v>2</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <f aca="false">SUM(G2:G3)</f>
-        <v>2</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <f aca="false">SUM(H2:H3)</f>
-        <v>2</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <f aca="false">SUM(I2:I3)</f>
+      <c r="F4" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H4" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="I4" s="4">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <f aca="false">SUM(J2:J3)</f>
-        <v>2</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <f aca="false">SUM(K2:K3)</f>
+      <c r="J4" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="K4" s="4">
+        <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <f aca="false">SUM(L2:L3)</f>
+      <c r="L4" s="4">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="M4" s="4">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="N4" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <f aca="false">SUM(M2:M3)</f>
-        <v>0</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <f aca="false">SUM(N2:N3)</f>
-        <v>0</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <f aca="false">SUM(B4:N4)</f>
-        <v>29.5</v>
+      <c r="O4" s="4">
+        <f>SUM(B4:N4)</f>
+        <v>42.5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultColWidth="10.47265625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="0" t="s">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="7">
         <v>45782</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" s="0" t="n">
-        <f aca="false">D2+E2</f>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <f t="shared" ref="F2:F17" si="0">D2+E2</f>
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="7">
         <v>45783</v>
       </c>
-      <c r="B3" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <f aca="false">D2+B3</f>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D17" si="1">D2+B3</f>
         <v>4</v>
       </c>
-      <c r="E3" s="0" t="n">
-        <f aca="false">E2+C3</f>
+      <c r="E3">
+        <f t="shared" ref="E3:E17" si="2">E2+C3</f>
         <v>4</v>
       </c>
-      <c r="F3" s="0" t="n">
-        <f aca="false">D3+E3</f>
+      <c r="F3">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
         <v>45789</v>
       </c>
-      <c r="B4" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <f aca="false">D3+B4</f>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="E4" s="0" t="n">
-        <f aca="false">E3+C4</f>
+      <c r="E4">
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="F4" s="0" t="n">
-        <f aca="false">D4+E4</f>
+      <c r="F4">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="7">
         <v>45790</v>
       </c>
-      <c r="B5" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <f aca="false">D4+B5</f>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="E5" s="0" t="n">
-        <f aca="false">E4+C5</f>
+      <c r="E5">
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="F5" s="0" t="n">
-        <f aca="false">D5+E5</f>
+      <c r="F5">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
         <v>45799</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6">
         <v>0</v>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <f aca="false">D5+B6</f>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="E6" s="0" t="n">
-        <f aca="false">E5+C6</f>
+      <c r="E6">
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="F6" s="0" t="n">
-        <f aca="false">D6+E6</f>
+      <c r="F6">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="7">
         <v>45804</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7">
         <v>1</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="0" t="n">
-        <f aca="false">D6+B7</f>
+      <c r="D7">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E7" s="0" t="n">
-        <f aca="false">E6+C7</f>
+      <c r="E7">
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="F7" s="0" t="n">
-        <f aca="false">D7+E7</f>
+      <c r="F7">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
         <v>45804</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8">
         <v>0</v>
       </c>
-      <c r="C8" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <f aca="false">D7+B8</f>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E8" s="0" t="n">
-        <f aca="false">E7+C8</f>
+      <c r="E8">
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="F8" s="0" t="n">
-        <f aca="false">D8+E8</f>
+      <c r="F8">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
         <v>45811</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9">
         <v>0</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9">
         <v>3</v>
       </c>
-      <c r="D9" s="0" t="n">
-        <f aca="false">D8+B9</f>
+      <c r="D9">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E9" s="0" t="n">
-        <f aca="false">E8+C9</f>
+      <c r="E9">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="F9" s="0" t="n">
-        <f aca="false">D9+E9</f>
+      <c r="F9">
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="7">
         <v>45813</v>
       </c>
-      <c r="C10" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="0" t="n">
-        <f aca="false">D9+B10</f>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E10" s="0" t="n">
-        <f aca="false">E9+C10</f>
+      <c r="E10">
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="F10" s="0" t="n">
-        <f aca="false">D10+E10</f>
+      <c r="F10">
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7">
         <v>45813</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="C11">
         <v>2.5</v>
       </c>
-      <c r="D11" s="0" t="n">
-        <f aca="false">D10+B11</f>
+      <c r="D11">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E11" s="0" t="n">
-        <f aca="false">E10+C11</f>
+      <c r="E11">
+        <f t="shared" si="2"/>
         <v>20.5</v>
       </c>
-      <c r="F11" s="0" t="n">
-        <f aca="false">D11+E11</f>
+      <c r="F11">
+        <f t="shared" si="0"/>
         <v>29.5</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
-      <c r="D12" s="0" t="n">
-        <f aca="false">D11+B12</f>
+      <c r="D12">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E12" s="0" t="n">
-        <f aca="false">E11+C12</f>
+      <c r="E12">
+        <f t="shared" si="2"/>
         <v>20.5</v>
       </c>
-      <c r="F12" s="0" t="n">
-        <f aca="false">D12+E12</f>
+      <c r="F12">
+        <f t="shared" si="0"/>
         <v>29.5</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="7"/>
-      <c r="D13" s="0" t="n">
-        <f aca="false">D12+B13</f>
+      <c r="D13">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E13" s="0" t="n">
-        <f aca="false">E12+C13</f>
+      <c r="E13">
+        <f t="shared" si="2"/>
         <v>20.5</v>
       </c>
-      <c r="F13" s="0" t="n">
-        <f aca="false">D13+E13</f>
+      <c r="F13">
+        <f t="shared" si="0"/>
         <v>29.5</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="7">
         <v>45818</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14">
         <v>6</v>
       </c>
-      <c r="D14" s="0" t="n">
-        <f aca="false">D13+B14</f>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="E14" s="0" t="n">
-        <f aca="false">E13+C14</f>
-        <v>20.5</v>
-      </c>
-      <c r="F14" s="0" t="n">
-        <f aca="false">D14+E14</f>
-        <v>35.5</v>
+      <c r="E14">
+        <f t="shared" si="2"/>
+        <v>23.5</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>38.5</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
-      <c r="D15" s="0" t="n">
-        <f aca="false">D14+B15</f>
+      <c r="D15">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="E15" s="0" t="n">
-        <f aca="false">E14+C15</f>
-        <v>20.5</v>
-      </c>
-      <c r="F15" s="0" t="n">
-        <f aca="false">D15+E15</f>
-        <v>35.5</v>
+      <c r="E15">
+        <f t="shared" si="2"/>
+        <v>23.5</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>38.5</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="7"/>
-      <c r="D16" s="0" t="n">
-        <f aca="false">D15+B16</f>
+      <c r="D16">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="E16" s="0" t="n">
-        <f aca="false">E15+C16</f>
-        <v>20.5</v>
-      </c>
-      <c r="F16" s="0" t="n">
-        <f aca="false">D16+E16</f>
-        <v>35.5</v>
+      <c r="E16">
+        <f t="shared" si="2"/>
+        <v>23.5</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>38.5</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
         <v>45820</v>
       </c>
-      <c r="B17" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="0" t="n">
-        <f aca="false">D16+B17</f>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="E17" s="0" t="n">
-        <f aca="false">E16+C17</f>
-        <v>22.5</v>
-      </c>
-      <c r="F17" s="0" t="n">
-        <f aca="false">D17+E17</f>
-        <v>39.5</v>
+      <c r="E17">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>42.5</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="7"/>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="7"/>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="7"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Préparer présentation/ Ajuster images Feuille de temps
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5011F503-4A3D-4076-8E3F-D917BFED5116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69C2DCA-7ACC-4D96-B20D-B00DC8F96F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille de temps" sheetId="1" r:id="rId1"/>
     <sheet name="Heures cumulées" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -350,6 +349,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-CA7F-4612-9881-F92DD63E748B}"/>
                 </c:ext>
@@ -381,6 +381,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-CA7F-4612-9881-F92DD63E748B}"/>
                 </c:ext>
@@ -1204,6 +1205,9 @@
                 <c:pt idx="12">
                   <c:v>45818</c:v>
                 </c:pt>
+                <c:pt idx="13">
+                  <c:v>45819</c:v>
+                </c:pt>
                 <c:pt idx="15">
                   <c:v>45820</c:v>
                 </c:pt>
@@ -1382,6 +1386,9 @@
                 <c:pt idx="12">
                   <c:v>45818</c:v>
                 </c:pt>
+                <c:pt idx="13">
+                  <c:v>45819</c:v>
+                </c:pt>
                 <c:pt idx="15">
                   <c:v>45820</c:v>
                 </c:pt>
@@ -1434,13 +1441,13 @@
                   <c:v>23.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>23.5</c:v>
+                  <c:v>26.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>23.5</c:v>
+                  <c:v>26.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>25.5</c:v>
+                  <c:v>28.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1560,6 +1567,9 @@
                 <c:pt idx="12">
                   <c:v>45818</c:v>
                 </c:pt>
+                <c:pt idx="13">
+                  <c:v>45819</c:v>
+                </c:pt>
                 <c:pt idx="15">
                   <c:v>45820</c:v>
                 </c:pt>
@@ -1612,13 +1622,13 @@
                   <c:v>38.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>38.5</c:v>
+                  <c:v>41.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>38.5</c:v>
+                  <c:v>41.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>42.5</c:v>
+                  <c:v>45.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1869,9 +1879,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>662760</xdr:colOff>
+      <xdr:colOff>670380</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
+      <xdr:rowOff>130995</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1905,9 +1915,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>266400</xdr:colOff>
+      <xdr:colOff>201630</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>11160</xdr:rowOff>
+      <xdr:rowOff>16875</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1948,7 +1958,7 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>75960</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148320</xdr:rowOff>
+      <xdr:rowOff>144510</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2299,7 +2309,8 @@
     <col min="2" max="2" width="11.44140625" customWidth="1"/>
     <col min="3" max="10" width="10.5546875" customWidth="1"/>
     <col min="11" max="11" width="10.77734375" customWidth="1"/>
-    <col min="12" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -2476,7 +2487,7 @@
         <v>9</v>
       </c>
       <c r="M4" s="4">
-        <f t="shared" si="0"/>
+        <f>SUM(M2:M3)</f>
         <v>4</v>
       </c>
       <c r="N4" s="4">
@@ -2806,18 +2817,23 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+      <c r="A15" s="7">
+        <v>45819</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
       <c r="D15">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>23.5</v>
+        <v>26.5</v>
       </c>
       <c r="F15">
         <f t="shared" si="0"/>
-        <v>38.5</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -2828,11 +2844,11 @@
       </c>
       <c r="E16">
         <f t="shared" si="2"/>
-        <v>23.5</v>
+        <v>26.5</v>
       </c>
       <c r="F16">
         <f t="shared" si="0"/>
-        <v>38.5</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -2851,11 +2867,11 @@
       </c>
       <c r="E17">
         <f t="shared" si="2"/>
-        <v>25.5</v>
+        <v>28.5</v>
       </c>
       <c r="F17">
         <f t="shared" si="0"/>
-        <v>42.5</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Régler bug affichage image/ préparer présentation
</commit_message>
<xml_diff>
--- a/Feuille_de_temps.xlsx
+++ b/Feuille_de_temps.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tompo\Cours\2024-2025\S2\S2.01\groupe19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37403C0C-8B54-4249-A96C-1EA3F5A1DB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFD1D81-990D-419E-9B62-508DDB244919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille de temps" sheetId="1" r:id="rId1"/>
@@ -448,7 +448,7 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>17</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>28.5</c:v>
@@ -639,10 +639,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'Feuille de temps'!$B$1:$I$1</c:f>
+              <c:f>'Feuille de temps'!$B$1:$N$1</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45782</c:v>
                 </c:pt>
@@ -666,16 +666,31 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>45811</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>45818</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>45819</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>45820</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Feuille de temps'!$B$2:$I$2</c:f>
+              <c:f>'Feuille de temps'!$B$2:$N$2</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
                 </c:pt>
@@ -690,6 +705,9 @@
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -763,10 +781,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'Feuille de temps'!$B$1:$I$1</c:f>
+              <c:f>'Feuille de temps'!$B$1:$N$1</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45782</c:v>
                 </c:pt>
@@ -790,16 +808,31 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>45811</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>45813</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>45818</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>45819</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>45820</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Feuille de temps'!$B$3:$I$3</c:f>
+              <c:f>'Feuille de temps'!$B$3:$N$3</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
                 </c:pt>
@@ -823,6 +856,21 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1270,7 +1318,7 @@
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>17</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1632,7 +1680,7 @@
                   <c:v>41.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>45.5</c:v>
+                  <c:v>43.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1883,9 +1931,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>670380</xdr:colOff>
+      <xdr:colOff>666570</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>130995</xdr:rowOff>
+      <xdr:rowOff>134805</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1919,9 +1967,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>89235</xdr:colOff>
+      <xdr:colOff>104475</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>16875</xdr:rowOff>
+      <xdr:rowOff>20685</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1953,16 +2001,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>259200</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>219195</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>148680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>75960</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>37860</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>144510</xdr:rowOff>
+      <xdr:rowOff>142605</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2356,7 +2404,7 @@
       <c r="M1" s="7">
         <v>45819</v>
       </c>
-      <c r="N1" s="6">
+      <c r="N1" s="7">
         <v>45820</v>
       </c>
       <c r="O1" s="1" t="s">
@@ -2391,12 +2439,10 @@
         <v>6</v>
       </c>
       <c r="M2" s="2"/>
-      <c r="N2" s="2">
-        <v>2</v>
-      </c>
+      <c r="N2" s="2"/>
       <c r="O2" s="2">
         <f>SUM(B2:N2)</f>
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
@@ -2501,11 +2547,11 @@
       </c>
       <c r="N4" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2">
         <f>SUM(B4:N4)</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -2864,15 +2910,12 @@
       <c r="A17" s="5">
         <v>45820</v>
       </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
       <c r="C17">
         <v>2</v>
       </c>
       <c r="D17">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E17">
         <f t="shared" si="2"/>
@@ -2880,7 +2923,7 @@
       </c>
       <c r="F17">
         <f t="shared" si="0"/>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>